<commit_message>
chore(boleta): actualizar plantilla boleta_template.xlsx
</commit_message>
<xml_diff>
--- a/backend/src/templates/boleta_template.xlsx
+++ b/backend/src/templates/boleta_template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <r>
       <rPr>
@@ -61,8 +61,7 @@
     <t>CALIFICACIÓN</t>
   </si>
   <si>
-    <t xml:space="preserve">PROMEDIO FINAL
-</t>
+    <t>PROMEDIO FINAL</t>
   </si>
   <si>
     <t>Extraordinario 01</t>
@@ -80,10 +79,16 @@
     <t>NOMBRE Y FIRMA DE LA DIRECTORA O DEL DIRECTOR:</t>
   </si>
   <si>
+    <t>HENRY JOSUE MAGAÑA NOVELO</t>
+  </si>
+  <si>
     <t>FIRMA DE ALUMNO</t>
   </si>
   <si>
     <t>LUGAR DE EXPEDICIÓN:</t>
+  </si>
+  <si>
+    <t>MÉRIDA, YUCATÁN</t>
   </si>
   <si>
     <t>FECHA DE EXPEDICIÓN:</t>
@@ -103,7 +108,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -182,6 +187,13 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -336,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -394,6 +406,9 @@
     <xf borderId="7" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="7" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -421,8 +436,8 @@
     </xf>
     <xf borderId="2" fillId="0" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -430,6 +445,9 @@
     <xf borderId="9" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="10" fillId="0" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -445,7 +463,7 @@
     <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="15" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="right" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
@@ -727,12 +745,12 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="4.5"/>
     <col customWidth="1" min="2" max="2" width="13.38"/>
-    <col customWidth="1" min="3" max="3" width="12.5"/>
-    <col customWidth="1" min="4" max="4" width="14.0"/>
-    <col customWidth="1" min="5" max="5" width="15.13"/>
-    <col customWidth="1" min="6" max="6" width="13.75"/>
-    <col customWidth="1" min="7" max="7" width="14.5"/>
-    <col customWidth="1" min="8" max="8" width="13.5"/>
+    <col customWidth="1" min="3" max="3" width="13.63"/>
+    <col customWidth="1" min="4" max="4" width="16.25"/>
+    <col customWidth="1" min="5" max="5" width="16.75"/>
+    <col customWidth="1" min="6" max="6" width="17.5"/>
+    <col customWidth="1" min="7" max="7" width="15.63"/>
+    <col customWidth="1" min="8" max="8" width="13.88"/>
     <col customWidth="1" min="9" max="9" width="3.25"/>
     <col customWidth="1" min="10" max="10" width="1.88"/>
     <col customWidth="1" min="11" max="12" width="9.38"/>
@@ -745,6 +763,8 @@
       <c r="F2" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
     </row>
     <row r="3" ht="32.25" customHeight="1">
       <c r="B3" s="2"/>
@@ -841,7 +861,7 @@
       <c r="M10" s="16"/>
       <c r="N10" s="17"/>
     </row>
-    <row r="11" ht="39.0" customHeight="1">
+    <row r="11" ht="38.25" customHeight="1">
       <c r="C11" s="20" t="s">
         <v>9</v>
       </c>
@@ -867,113 +887,115 @@
       </c>
     </row>
     <row r="12" ht="30.0" customHeight="1">
-      <c r="C12" s="20" t="s">
+      <c r="C12" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="23" t="str">
+      <c r="D12" s="24" t="str">
         <f t="array" ref="D12">IFERROR(VLOOKUP($F$5, INDIRECT("'" &amp; $O$4 &amp; "'!C:I"), 7, FALSE), "")</f>
         <v/>
       </c>
       <c r="E12" s="15"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="24"/>
-      <c r="J12" s="25" t="s">
+      <c r="H12" s="25"/>
+      <c r="J12" s="26" t="s">
         <v>11</v>
       </c>
       <c r="K12" s="15"/>
-      <c r="L12" s="24"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="24"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="25"/>
     </row>
     <row r="13" ht="23.25" customHeight="1">
-      <c r="C13" s="27"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="J13" s="29" t="s">
+      <c r="C13" s="28"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="J13" s="30" t="s">
         <v>12</v>
       </c>
       <c r="K13" s="15"/>
-      <c r="L13" s="24"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="24"/>
+      <c r="L13" s="25"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="25"/>
     </row>
     <row r="14" ht="32.25" customHeight="1">
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
-      <c r="J14" s="25" t="s">
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="J14" s="26" t="s">
         <v>14</v>
       </c>
       <c r="K14" s="15"/>
-      <c r="L14" s="24"/>
-      <c r="M14" s="32"/>
-      <c r="N14" s="24"/>
+      <c r="L14" s="25"/>
+      <c r="M14" s="33"/>
+      <c r="N14" s="25"/>
     </row>
     <row r="16" ht="7.5" customHeight="1"/>
     <row r="17">
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="F17" s="34"/>
+      <c r="F17" s="35" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="18">
-      <c r="J18" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="K18" s="36"/>
-      <c r="L18" s="36"/>
-      <c r="M18" s="36"/>
-      <c r="N18" s="36"/>
-      <c r="O18" s="37"/>
+      <c r="J18" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="K18" s="37"/>
+      <c r="L18" s="37"/>
+      <c r="M18" s="37"/>
+      <c r="N18" s="37"/>
+      <c r="O18" s="38"/>
     </row>
     <row r="19">
-      <c r="C19" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="E19" s="39"/>
-      <c r="H19" s="39"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="41"/>
-      <c r="L19" s="41"/>
-      <c r="M19" s="41"/>
-      <c r="N19" s="41"/>
-      <c r="O19" s="42"/>
+      <c r="C19" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>19</v>
+      </c>
+      <c r="H19" s="41"/>
+      <c r="J19" s="42"/>
+      <c r="K19" s="43"/>
+      <c r="L19" s="43"/>
+      <c r="M19" s="43"/>
+      <c r="N19" s="43"/>
+      <c r="O19" s="44"/>
     </row>
     <row r="20">
-      <c r="J20" s="43"/>
+      <c r="J20" s="45"/>
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
       <c r="N20" s="10"/>
-      <c r="O20" s="44"/>
+      <c r="O20" s="46"/>
     </row>
     <row r="21">
-      <c r="C21" s="38" t="s">
-        <v>18</v>
-      </c>
-      <c r="E21" s="45">
-        <v>46242.0</v>
-      </c>
-      <c r="H21" s="39"/>
-      <c r="J21" s="46"/>
-      <c r="K21" s="47"/>
-      <c r="L21" s="47"/>
-      <c r="M21" s="47"/>
-      <c r="N21" s="47"/>
-      <c r="O21" s="48"/>
+      <c r="C21" s="39" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="47"/>
+      <c r="H21" s="41"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="49"/>
+      <c r="N21" s="49"/>
+      <c r="O21" s="50"/>
     </row>
     <row r="22">
-      <c r="G22" s="38" t="s">
-        <v>19</v>
+      <c r="G22" s="39" t="s">
+        <v>21</v>
       </c>
       <c r="J22" s="10"/>
       <c r="K22" s="10"/>
@@ -991,13 +1013,10 @@
       <c r="O23" s="10"/>
     </row>
     <row r="24">
-      <c r="B24" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
+      <c r="B24" s="51" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="52"/>
       <c r="I24" s="10"/>
       <c r="J24" s="10"/>
       <c r="K24" s="10"/>
@@ -1955,20 +1974,20 @@
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="D12:H12"/>
-    <mergeCell ref="F2:J2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="F5:K5"/>
     <mergeCell ref="M5:P5"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="M14:N14"/>
-    <mergeCell ref="F17:K17"/>
     <mergeCell ref="J18:O18"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="E21:G21"/>
-    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="F17:K17"/>
+    <mergeCell ref="C24:H24"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="J9:M9"/>
     <mergeCell ref="J10:M10"/>

</xml_diff>